<commit_message>
fix: parse quantities after specification units
</commit_message>
<xml_diff>
--- a/docs/order-moa-real-order-test-cases.xlsx
+++ b/docs/order-moa-real-order-test-cases.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>성공 9 / 별칭_필요 2 / 수량_확인 2 / 단위_확인 2 / 단가_미등록 1 / 오매칭_위험 2</t>
+          <t>성공 10 / 별칭_필요 2 / 수량_확인 2 / 단위_확인 2 / 단가_미등록 1 / 오매칭_위험 1</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr"/>
@@ -2104,17 +2104,17 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>의도는 2봉인데 첫 숫자 '1'(1kg의 1)을 수량으로 잡을 위험</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>오매칭_위험</t>
+          <t>규격 숫자(1kg)는 제외하고 수량 2봉 채택</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>성공</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>파서가 첫 숫자를 수량으로 사용 — 규격 숫자와 수량 숫자 구분 없음</t>
+          <t>개선 1차(2026-07-02) 적용: 수량단위 결합 숫자 &gt; 단독 숫자 &gt; 측정단위(kg/g/L/ml) 결합 숫자 우선순위</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr"/>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>숫자+중량단위(kg/L/g) 결합은 규격 후보로 강등, 마지막 독립 숫자를 수량 우선</t>
+          <t>숫자+중량단위(kg/L/g/ml) 결합은 우선순위 강등(수량단위&gt;단독&gt;측정단위)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: require confirmation for ambiguous product matches
</commit_message>
<xml_diff>
--- a/docs/order-moa-real-order-test-cases.xlsx
+++ b/docs/order-moa-real-order-test-cases.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -53,22 +53,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E4DFEC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,10 +93,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -116,9 +111,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -486,11 +478,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,25 +500,115 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>expectedSummary</t>
+          <t>원본</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>{"성공": 12, "별칭_필요": 2, "수량_확인": 2, "단위_확인": 0, "단가_미등록": 1, "오매칭_위험": 1}</t>
+          <t>실사용 이카운트 판매조회 엑셀(식당납품, 191건/거래처 12곳/고유 품목 71종)에서 패턴만 일반화</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>비고</t>
+          <t>익명화</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>실거래처명/공급사명/브랜드명은 일반화. 실제 단가/금액 미사용.</t>
-        </is>
+          <t>실거래처명→A식당~E마트 가명, 공급사명(괄호 안 상호)→'공급사S'류 일반화, 브랜드명→(브랜드) 표기, 실단가/실금액 미사용(테스트용 임의값), 전화/주소/사업자번호 원본에 없음·미수록</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>품목 수</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>발주문장 수</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>예상 상태: 성공</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>예상 상태: 후보_확인</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>예상 상태: 별칭_필요</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>예상 상태: 수량_확인</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>예상 상태: 단위_확인</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>예상 상태: 단가_미등록</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>예상 상태: 오매칭_위험</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -543,19 +625,19 @@
   <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -565,7 +647,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>기준단위</t>
+          <t>기본단위</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -575,12 +657,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>판매단가</t>
+          <t>테스트 단가</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>기준매입단가</t>
+          <t>기준 매입단가</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -1437,20 +1519,20 @@
   <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -1465,12 +1547,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>기대 상태</t>
+          <t>예상 상태</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>기대 내용</t>
+          <t>예상 결과</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -1490,17 +1572,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>t01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>A식당</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>세척숙주 3박스
 청경채 2박스
@@ -1512,31 +1594,31 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>3라인 전부 매칭·수량 확정</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>품목명/별칭 포함매칭 + 아라비아 숫자 + 단위 사전</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>t02</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>C반찬</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>취나물 2봉
 깍둑단무지 3개</t>
@@ -1547,65 +1629,65 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>별칭으로 건취나물/단무지 매칭</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>등록 별칭 매칭</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>t03</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>B분식</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>숙주 3박스</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>오매칭_위험</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>세척숙주(BOX)로 가야 하나 '숙주' 토큰이 rp01/rp02 둘 다 포함 → 등록 순서에 따라 결정</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>포함매칭이 첫 일치 품목 반환(다중 후보 미제시)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>후보_확인</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>'숙주' 토큰이 rp01/rp02 둘 다 포함 → 후보 확인 후 사용자가 최종 선택</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>개선 3차(2026-07-06) 적용: 다중 후보면 후보 목록 표시 + 확정 차단</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>t04</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>A식당</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>무 2개</t>
         </is>
@@ -1615,31 +1697,31 @@
           <t>별칭_필요</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>'무'는 1글자라 포함매칭 제외 → 품목명 '무 [20kg 국산]'과 정확일치 실패</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>1글자 토큰은 정확일치만 허용 → 별칭 '무' 등록 후 매칭</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>t05</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>A식당</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>무순 3개</t>
         </is>
@@ -1649,101 +1731,101 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>무순 [EA] 매칭(2글자 포함매칭)</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>'무순'은 2글자라 포함매칭 허용</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>t06</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>A식당</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>감자 조금
 대파 두 단</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>수량_확인</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>품목 매칭되나 수량 null → 확정 차단</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>모호 표현('조금')·한글 수사('두')</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>t07</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>D마트</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>계란 특 두판
 배추 한망</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>수량_확인</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>계란[특]/배추(5입) 매칭 여부 + 한글 수사</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>'두판','한망'은 수량 불확실. '계란 특' 토큰은 '계란' 별칭으로 흡수</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>t08</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>B분식</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>○○떡 5봉</t>
         </is>
@@ -1753,31 +1835,31 @@
           <t>별칭_필요</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>브랜드 호칭(○○떡)은 미매칭 → 품목 지정 후 별칭 등록으로 해결되는지 확인</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>브랜드명 호칭은 품목명/별칭 사전에 없음 — 실데이터에서 브랜드로 부르는 품목 존재(가명화)</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>t09</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>C반찬</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>치커리 2, 양상추 1, 부추 3단</t>
         </is>
@@ -1787,65 +1869,65 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>쉼표 분리 3라인, 단위 일부 생략(base_unit 추정)</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>한 줄 다품목 분리 + 숫자만 수량</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>t10</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>E카페</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>세척숙주 1박스</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>단가_미등록</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>매칭되지만 E카페 단가 미등록 → 0원+경고+즉석 저장</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>customer_prices 미등록 조합</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>t11</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>B분식</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>청양고추 1kg 2봉</t>
         </is>
@@ -1855,31 +1937,31 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>규격 숫자(1kg)는 제외하고 수량 2봉 채택</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>개선 1차(2026-07-02) 적용: 수량단위 결합 숫자 &gt; 단독 숫자 &gt; 측정단위(kg/g/L/ml) 결합 숫자 우선순위</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>t12</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>D마트</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>소불고기 2키로</t>
         </is>
@@ -1889,31 +1971,31 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>품목 매칭, '키로'는 kg로 표준화</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>개선 2차(2026-07-06) 적용: 키로/킬로 계열을 kg로 표준화</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>t13</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>D마트</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>메추리알 2봉</t>
         </is>
@@ -1923,31 +2005,31 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>매칭+수량 2. 품목명 안 '20EA' 숫자는 발주문장에 없어 영향 없음</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>이름 내 숫자는 발주 원문이 아니면 무해</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>t14</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>D마트</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>락스 2개, 비닐 3장</t>
         </is>
@@ -1957,31 +2039,31 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>공산품 매칭. '장' 단위 직접 인식</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>개선 2차(2026-07-06) 적용: 장/마리/모/봉지 단위 추가</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>t15</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>A식당</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>알배추 2박스</t>
         </is>
@@ -1991,31 +2073,31 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>알배기(알배추) 별칭 매칭</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>괄호 병기 호칭을 별칭으로 흡수</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>t16</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>C반찬</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>쪽파 2봉이랑 두부 3개 부탁해요</t>
         </is>
@@ -2025,31 +2107,31 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>연결어 분리 + 군말 제거 → 깐쪽파/팩두부</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>'이랑' 분리 + 별칭</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>t17</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>A식당</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>국거리 1팩</t>
         </is>
@@ -2059,31 +2141,31 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>우(국거리) 포함매칭</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>별칭 '국거리'</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>t18</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>B분식</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>양파1망</t>
         </is>
@@ -2093,18 +2175,18 @@
           <t>성공</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>공백 없어도 숫자/단위 분리</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>정규식이 공백 없이도 숫자+단위 추출</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2117,62 +2199,113 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>구분</t>
+          <t>분류</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>대상</t>
+          <t>예시</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>내용</t>
+          <t>권장 처리</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>단가 미등록</t>
+          <t>규격 숫자 vs 수량 숫자 구분 없음</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>E카페</t>
+          <t>청양고추 1kg 2봉 → 수량 1로 오인</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>rp01 · E카페는 세척숙주 단가 미등록 → 0원+즉석 저장 테스트</t>
+          <t>숫자+중량단위(kg/L/g/ml) 결합은 우선순위 강등(수량단위&gt;단독&gt;측정단위) / 적용 완료(2026-07-02, order-parser.ts pickQuantityCluster)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>단가 미등록</t>
+          <t>동일 토큰 다중 품목 시 첫 매칭 반환</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>A식당</t>
+          <t>'숙주' → 세척숙주 vs 숙주(1kg) 중 등록순</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>rp07 · 햇감자 전 거래처 단가 미등록(시세 변동) → 즉석 입력 흐름</t>
+          <t>다중 후보면 사용자 선택 드롭다운 우선 노출(오매칭보다 확인이 안전) / 적용 완료(2026-07-06, 후보 목록 표시 + 선택 전 확정 차단)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1글자 품목(무·파 등) 정확일치만 허용</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>'무 2개' 미매칭</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>현행 유지가 안전(단무지 오매칭 방지). 대신 별칭 등록 안내 문구 강화</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>단위 사전 부족</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>키로, 장, 마리, 모</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>단위 사전에 키로/키로그람/장/마리/모 추가 / 적용 완료(2026-07-06, 키로/킬로→kg 표준화 + 장/마리/모/봉지 인식)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>규격 포함 품목명 표기 표준</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>품목명(규격) [단위] 혼재</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>1차는 이름에 포함 유지(스펙 §10.3), 표기 가이드만 문서화</t>
         </is>
       </c>
     </row>
@@ -2187,14 +2320,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2205,7 +2338,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>이슈</t>
+          <t>문제</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -2215,7 +2348,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>개선 아이디어</t>
+          <t>아이디어</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -2223,6 +2356,123 @@
           <t>상태</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>규격 숫자 vs 수량 숫자 구분 없음</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>청양고추 1kg 2봉 → 수량 1로 오인</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>숫자+중량단위(kg/L/g/ml) 결합은 우선순위 강등(수량단위&gt;단독&gt;측정단위)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>적용 완료(2026-07-02, order-parser.ts pickQuantityCluster)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>동일 토큰 다중 품목 시 첫 매칭 반환</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>'숙주' → 세척숙주 vs 숙주(1kg) 중 등록순</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>다중 후보면 사용자 선택 드롭다운 우선 노출(오매칭보다 확인이 안전)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>적용 완료(2026-07-06, 후보 목록 표시 + 선택 전 확정 차단)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>1글자 품목(무·파 등) 정확일치만 허용</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>'무 2개' 미매칭</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>현행 유지가 안전(단무지 오매칭 방지). 대신 별칭 등록 안내 문구 강화</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>단위 사전 부족</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>키로, 장, 마리, 모</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>단위 사전에 키로/키로그람/장/마리/모 추가</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>적용 완료(2026-07-06, 키로/킬로→kg 표준화 + 장/마리/모/봉지 인식)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>규격 포함 품목명 표기 표준</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>품목명(규격) [단위] 혼재</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1차는 이름에 포함 유지(스펙 §10.3), 표기 가이드만 문서화</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>